<commit_message>
v2 of box profile with new componets and format. updated some docs
</commit_message>
<xml_diff>
--- a/data/baseball_scp_master.xlsx
+++ b/data/baseball_scp_master.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -522,10 +522,14 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-bowman-chrome-sapphire</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-chrome-sapphire</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G22994</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -550,11 +554,7 @@
           <t>2018 Bowman Sterling</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-bowman-sterling</t>
-        </is>
-      </c>
+      <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
@@ -735,10 +735,14 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-panini-prizm</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/basketball-cards-2018-panini-prizm</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G2068</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -746,11 +750,7 @@
           <t>2018 Panini Prizm Draft Picks</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-panini-prizm-draft-picks</t>
-        </is>
-      </c>
+      <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
@@ -844,11 +844,7 @@
           <t>2018 Topps Archives Signature Series Active Player Edition</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-archives-signature-series-active-player-edition</t>
-        </is>
-      </c>
+      <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
@@ -857,11 +853,7 @@
           <t>2018 Topps Archives Signature Series Retired Player Edition</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-archives-signature-series-retired-player-edition</t>
-        </is>
-      </c>
+      <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
@@ -938,11 +930,7 @@
           <t>2018 Topps Definitive Collection</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-definitive-collection</t>
-        </is>
-      </c>
+      <c r="B31" s="3" t="n"/>
       <c r="C31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
@@ -951,11 +939,7 @@
           <t>2018 Topps Diamond Icons</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-diamond-icons</t>
-        </is>
-      </c>
+      <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
@@ -964,11 +948,7 @@
           <t>2018 Topps Dynasty</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-dynasty</t>
-        </is>
-      </c>
+      <c r="B33" s="3" t="n"/>
       <c r="C33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1079,11 +1059,7 @@
           <t>2018 Topps Heritage High Number</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2018-topps-heritage-high-number</t>
-        </is>
-      </c>
+      <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
@@ -1236,6 +1212,23 @@
       <c r="C49" s="3" t="inlineStr">
         <is>
           <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G23347</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2018 Bowman Sterling (Continuity)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2018-bowman-sterling-continuity</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G22545</t>
         </is>
       </c>
     </row>
@@ -1315,11 +1308,7 @@
           <t>2019 Bowman Chrome X</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-bowman-chrome-x</t>
-        </is>
-      </c>
+      <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
@@ -1464,11 +1453,7 @@
           <t>2019 Leaf Metal Babe Ruth Collection</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-leaf-metal-babe-ruth-collection</t>
-        </is>
-      </c>
+      <c r="B13" s="3" t="n"/>
       <c r="C13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1477,11 +1462,7 @@
           <t>2019 Leaf Metal Perfect Game All-American</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-leaf-metal-perfect-game-all-american</t>
-        </is>
-      </c>
+      <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1490,11 +1471,7 @@
           <t>2019 Onyx Vintage Collection</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-onyx-vintage-collection</t>
-        </is>
-      </c>
+      <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1573,10 +1550,14 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-panini-leather-and-lumber</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2019-panini-leather-&amp;-lumber</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G23691</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1703,11 +1684,7 @@
           <t>2019 Topps Archives Signature Series Active Player Edition</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-archives-signature-series-active-player-edition</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1716,11 +1693,7 @@
           <t>2019 Topps Archives Signature Series Retired Player Edition</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-archives-signature-series-retired-player-edition</t>
-        </is>
-      </c>
+      <c r="B29" s="3" t="n"/>
       <c r="C29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1831,11 +1804,7 @@
           <t>2019 Topps Definitive Collection</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-definitive-collection</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1844,11 +1813,7 @@
           <t>2019 Topps Diamond Icons</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-diamond-icons</t>
-        </is>
-      </c>
+      <c r="B37" s="3" t="n"/>
       <c r="C37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1857,11 +1822,7 @@
           <t>2019 Topps Dynasty</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-dynasty</t>
-        </is>
-      </c>
+      <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1991,10 +1952,14 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-holiday</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-holiday-mega-box</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G24037</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2019,11 +1984,7 @@
           <t>2019 Topps Luminaries</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2019-topps-luminaries</t>
-        </is>
-      </c>
+      <c r="B48" s="2" t="n"/>
       <c r="C48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
@@ -2238,11 +2199,7 @@
           <t>2020 Bowman Chrome X</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-bowman-chrome-x</t>
-        </is>
-      </c>
+      <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
@@ -2287,10 +2244,14 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-bowman-sapphire</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2020-bowman-chrome-prospects-sapphire</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G24363</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2587,11 +2548,7 @@
           <t>2020 Topps Allen &amp; Ginter X</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-allen-&amp;-ginter-x</t>
-        </is>
-      </c>
+      <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
@@ -2617,11 +2574,7 @@
           <t>2020 Topps Archives Signature Series Active Player Edition</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-archives-signature-series-active-player-edition</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2630,11 +2583,7 @@
           <t>2020 Topps Archives Signature Series Retired Player Edition</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-archives-signature-series-retired-player-edition</t>
-        </is>
-      </c>
+      <c r="B29" s="3" t="n"/>
       <c r="C29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
@@ -2711,11 +2660,7 @@
           <t>2020 Topps Chrome Ben Baller Edition</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-chrome-ben-baller-edition</t>
-        </is>
-      </c>
+      <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2741,11 +2686,7 @@
           <t>2020 Topps Chrome Celebration of the Decades</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-chrome-celebration-of-the-decades</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2822,11 +2763,7 @@
           <t>2020 Topps Definitive Collection</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-definitive-collection</t>
-        </is>
-      </c>
+      <c r="B41" s="3" t="n"/>
       <c r="C41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2835,11 +2772,7 @@
           <t>2020 Topps Diamond Icons</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-diamond-icons</t>
-        </is>
-      </c>
+      <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2882,11 +2815,7 @@
           <t>2020 Topps Five Star</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-five-star-autographs</t>
-        </is>
-      </c>
+      <c r="B45" s="3" t="n"/>
       <c r="C45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2997,11 +2926,7 @@
           <t>2020 Topps Luminaries</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2020-topps-luminaries</t>
-        </is>
-      </c>
+      <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
@@ -3148,11 +3073,7 @@
           <t>2021 Bowman Chrome X</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-bowman-chrome-x</t>
-        </is>
-      </c>
+      <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -3265,10 +3186,14 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-bowman%27s-best</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2021-bowman%e2%80%99s-best</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G48407</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3599,11 +3524,7 @@
           <t>2021 Topps Archives Signature Series Active Player Edition</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-topps-archives-signature-series-active-player-edition</t>
-        </is>
-      </c>
+      <c r="B33" s="3" t="n"/>
       <c r="C33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
@@ -3663,11 +3584,7 @@
           <t>2021 Topps Brooklyn Collection</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-topps-brooklyn-collection</t>
-        </is>
-      </c>
+      <c r="B37" s="3" t="n"/>
       <c r="C37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -3967,10 +3884,14 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-topps-holiday</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2021-topps-holiday-mega-box</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G47948</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4012,11 +3933,7 @@
           <t>2021 Topps Luminaries</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-topps-luminaries</t>
-        </is>
-      </c>
+      <c r="B58" s="2" t="n"/>
       <c r="C58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
@@ -4127,11 +4044,7 @@
           <t>2021 Topps Transcendent Collection Hall of Fame Edition</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2021-topps-transcendent-collection-hall-of-fame-edition</t>
-        </is>
-      </c>
+      <c r="B65" s="3" t="n"/>
       <c r="C65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
@@ -4295,11 +4208,7 @@
           <t>2022 Bowman Chrome Sapphire Edition</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-bowman-chrome-sapphire</t>
-        </is>
-      </c>
+      <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
@@ -4308,11 +4217,7 @@
           <t>2022 Bowman Chrome X</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-bowman-chrome-x</t>
-        </is>
-      </c>
+      <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4398,11 +4303,7 @@
           <t>2022 Bowman Transcendent Collection</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-bowman-transcendent-collection</t>
-        </is>
-      </c>
+      <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
@@ -4479,11 +4380,7 @@
           <t>2022 Finest Flashbacks</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-finest-flashbacks</t>
-        </is>
-      </c>
+      <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
@@ -4492,11 +4389,7 @@
           <t>2022 Leaf Lumber</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-leaf-lumber</t>
-        </is>
-      </c>
+      <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
@@ -4505,11 +4398,7 @@
           <t>2022 Leaf Vivid</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-leaf-vivid</t>
-        </is>
-      </c>
+      <c r="B19" s="3" t="n"/>
       <c r="C19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
@@ -4807,11 +4696,7 @@
           <t>2022 Topps Allen &amp; Ginter X</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-allen-&amp;-ginter-x</t>
-        </is>
-      </c>
+      <c r="B37" s="3" t="n"/>
       <c r="C37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -5109,11 +4994,7 @@
           <t>2022 Topps Definitive Collection</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-definitive-collection</t>
-        </is>
-      </c>
+      <c r="B55" s="3" t="n"/>
       <c r="C55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
@@ -5122,11 +5003,7 @@
           <t>2022 Topps Diamond Icons</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-diamond-icons</t>
-        </is>
-      </c>
+      <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
@@ -5135,11 +5012,7 @@
           <t>2022 Topps Dynasty</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-dynasty</t>
-        </is>
-      </c>
+      <c r="B57" s="3" t="n"/>
       <c r="C57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
@@ -5318,11 +5191,7 @@
           <t>2022 Topps Luminaries</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-luminaries</t>
-        </is>
-      </c>
+      <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
@@ -5331,11 +5200,7 @@
           <t>2022 Topps Mini</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-mini</t>
-        </is>
-      </c>
+      <c r="B69" s="3" t="n"/>
       <c r="C69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
@@ -5412,11 +5277,7 @@
           <t>2022 Topps Sterling</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2022-topps-sterling</t>
-        </is>
-      </c>
+      <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
@@ -5861,11 +5722,7 @@
           <t>2023 Topps 1st Edition</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-1st-edition</t>
-        </is>
-      </c>
+      <c r="B20" s="2" t="n"/>
       <c r="C20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
@@ -5891,11 +5748,7 @@
           <t>2023 Topps Allen &amp; Ginter X</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-allen-&amp;-ginter-x</t>
-        </is>
-      </c>
+      <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
@@ -6059,10 +5912,14 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-chrome-logofractor</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-chrome-logofractor-autograph</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G69780</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -6138,11 +5995,7 @@
           <t>2023 Topps Definitive Collection</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-definitive-collection</t>
-        </is>
-      </c>
+      <c r="B37" s="3" t="n"/>
       <c r="C37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -6153,10 +6006,14 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-diamond-icons</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-diamond-icons-autograph</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70308</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -6283,11 +6140,7 @@
           <t>2023 Topps Luminaries</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-luminaries</t>
-        </is>
-      </c>
+      <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
@@ -6347,11 +6200,7 @@
           <t>2023 Topps Sterling</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-sterling</t>
-        </is>
-      </c>
+      <c r="B50" s="2" t="n"/>
       <c r="C50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
@@ -6377,11 +6226,7 @@
           <t>2023 Topps Transcendent Collection</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-transcendent-collection</t>
-        </is>
-      </c>
+      <c r="B52" s="2" t="n"/>
       <c r="C52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
@@ -6426,10 +6271,14 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-world-baseball-classic</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr"/>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2023-topps-world-classic</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G67599</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -6524,11 +6373,7 @@
           <t>2024 Bowman Chrome Sapphire Edition</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-bowman-chrome-sapphire</t>
-        </is>
-      </c>
+      <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
@@ -6745,587 +6590,575 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2024 Stadium Club</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-stadium-club</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G68643</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G68643</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Allen &amp; Ginter</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-allen-%26-ginter</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75037</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Allen &amp; Ginter</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-allen-%26-ginter</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75037</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Allen &amp; Ginter X</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-allen-%26-ginter-x</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76367</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Allen &amp; Ginter X</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-allen-%26-ginter-x</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76367</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Archives</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-archives</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77385</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Archives</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-archives</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77385</t>
-        </is>
-      </c>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Archives Signature Series Active Player Edition</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Archives Signature Series Active Player Edition</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-archives-signature-series-active-player-edition</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Archives Signature Series Retired Player Edition</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Archives Signature Series Retired Player Edition</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-archives-signature-series-retired-player-edition</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Big League</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-big-league-baseball</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G69605</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Big League</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-big-league</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Black &amp; White</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-black-and-white</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77662</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Black &amp; White</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-black-and-white</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77662</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Brooklyn Collection</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-brooklyn-collection</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76577</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Brooklyn Collection</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-brooklyn-collection</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76577</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G71691</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G71691</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Black</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-black</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70272</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome Black</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-black</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70272</t>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Cosmic</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-cosmic-chrome</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74648</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome Cosmic</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-cosmic-chrome</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74648</t>
-        </is>
-      </c>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Logofractor Edition</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome Logofractor Edition</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-logofractor</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-sapphire</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74676</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome Sapphire Edition</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-sapphire</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74676</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Update</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-update</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75594</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome Update</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-update</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75594</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Chrome Update Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-sapphire-update</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76503</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Chrome Update Sapphire Edition</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-chrome-update-sapphire</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Definitive Collection</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Definitive Collection</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-definitive-collection</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Diamond Icons</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Diamond Icons</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-diamond-icons</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Dynamic Duals</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Dynamic Duals</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-dynamic-duals</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Dynasty</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-dynasty</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G83364</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Dynasty</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-dynasty</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G83364</t>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Five Star</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-five-star-autograph</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74344</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Five Star</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-five-star-autographs</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Gilded Collection</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-gilded-collection</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75879</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Gilded Collection</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-gilded-collection</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75879</t>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Heritage</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-heritage</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70086</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Heritage</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-heritage</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70086</t>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Heritage Mini</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-heritage-mini</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70762</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Heritage Mini</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-heritage-mini</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G70762</t>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Holiday</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-holiday</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75656</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Holiday</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-holiday</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75656</t>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Inception</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-inception</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G82837</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Inception</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-inception</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G82837</t>
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Japan Edition</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-japan-edition</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91485</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Japan Edition</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-japan-edition</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91485</t>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Luminaries</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-luminaries</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77418</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Luminaries</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-luminaries</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77418</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Museum Collection</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-museum-collection</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G72321</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Museum Collection</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-museum-collection</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G72321</t>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Pristine</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-pristine</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G73473</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Pristine</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-pristine</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G73473</t>
-        </is>
-      </c>
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Sterling</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n"/>
+      <c r="C48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Sterling</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-sterling</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Tier One</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-tier-one</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G71518</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Tier One</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-tier-one</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G71518</t>
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Transcendent Collection</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-transcendent-collection</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77951</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Transcendent Collection</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-transcendent-collection</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G77951</t>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Tribute</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-tribute</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G69496</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Tribute</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-tribute</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G69496</t>
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2024 Topps Triple Threads</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-triple-threads</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76710</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>2024 Topps Triple Threads</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-triple-threads</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G76710</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2024 Topps Update</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-update</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74468</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>2024 Topps Update</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-update</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G74468</t>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2024 Topps Stadium Club</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2024-topps-stadium-club</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G75167</t>
         </is>
       </c>
     </row>
@@ -7405,11 +7238,7 @@
           <t>2025 Bowman Chrome Sapphire Edition</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-bowman-chrome-sapphire</t>
-        </is>
-      </c>
+      <c r="B4" s="2" t="n"/>
       <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
@@ -7592,484 +7421,472 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>2025 Stadium Club</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-stadium-club</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G78872</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G78872</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Allen &amp; Ginter</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-allen-and-ginter</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89225</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Allen &amp; Ginter</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-allen-and-ginter</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89225</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Allen &amp; Ginter X</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-allen-%26-ginter-x</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G90445</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Allen &amp; Ginter X</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-allen-%26-ginter-x</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G90445</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps All-Star Game</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-all-star-game</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G84149</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps All-Star Game</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-all-star-game</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G84149</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Archives</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-archives</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89499</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Archives</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-archives</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89499</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Archives Signature Series Active Player Edition</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Archives Signature Series Active Player Edition</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-archives-signature-series-active-player-edition</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Black &amp; White</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-black-and-white</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89768</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Black &amp; White</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-black-and-white</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89768</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G83992</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G83992</t>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Black</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-black</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G80820</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Black</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-black</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G80820</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Cosmic</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-cosmic-chrome</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89637</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Cosmic</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-cosmic-chrome</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89637</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Logofractor Edition</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-logofractor</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G86144</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Logofractor Edition</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-logofractor</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G86144</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Platinum</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-platinum</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G96493</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Platinum</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-platinum</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G96493</t>
-        </is>
-      </c>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Sapphire Edition</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-sapphire</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Update</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-update</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89472</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Update</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-update</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89472</t>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Chrome Update Sapphire Edition</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-sapphire-update</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G90439</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Chrome Update Sapphire Edition</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-chrome-update-sapphire</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Definitive Collection</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Definitive Collection</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-definitive-collection</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Diamond Icons</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-diamond-icons</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G88210</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Diamond Icons</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-diamond-icons</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G88210</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Dynamic Duals</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-dynamic-duals</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G83727</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Dynamic Duals</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-dynamic-duals</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G83727</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Five Star</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-five-star</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89889</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Five Star</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-five-star</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G89889</t>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Gilded Collection</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-gilded-collection</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91369</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Gilded Collection</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-gilded-collection</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91369</t>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Heritage</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-heritage</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G80830</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Heritage</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-heritage</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G80830</t>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Holiday</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-holiday</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G88244</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Holiday</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-holiday</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G88244</t>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Museum Collection</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-museum-collection</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91138</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Museum Collection</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-museum-collection</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91138</t>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Pristine</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-pristine</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G90880</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Pristine</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-pristine</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G90880</t>
-        </is>
-      </c>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Sterling</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n"/>
+      <c r="C40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Sterling</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-sterling</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Tier One</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-tier-one</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G86239</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Tier One</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-tier-one</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G86239</t>
-        </is>
-      </c>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Transcendent Collection</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n"/>
+      <c r="C42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Transcendent Collection</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-transcendent-collection</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2025 Topps Tribute</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-tribute</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G80518</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>2025 Topps Tribute</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-tribute</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G80518</t>
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2025 Topps Update</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-update</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G87704</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>2025 Topps Update</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-update</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G87704</t>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025 Topps Stadium Club</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/console/baseball-cards-2025-topps-stadium-club</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.sportscardspro.com/price-guide/download-custom?t=7f389d8e7c6dbb986abeec5f5789ac4a0a4cac15&amp;console-uids=G91593</t>
         </is>
       </c>
     </row>
@@ -8200,11 +8017,7 @@
           <t>2026 Topps Japan Edition</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sportscardspro.com/console/baseball-cards-2026-topps-japan-edition</t>
-        </is>
-      </c>
+      <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>